<commit_message>
Add Oracle Q1 FY27 filings and populate EV bridge
Fetched the 10-Q for the quarter ended Aug 31, 2026 and the FY26 10-K
from EDGAR into filings/ORCL/, and wrote the Oracle EV bridge into
templates/TradingComps.xlsx with a source note on every cell.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012dLLbpnyoNB7T2efRSv67L
</commit_message>
<xml_diff>
--- a/templates/TradingComps.xlsx
+++ b/templates/TradingComps.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,11 @@
     <font>
       <name val="Aptos"/>
       <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -70,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -78,6 +83,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -152,6 +158,99 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Cash and cash equivalents
+pg 4
+Marketable securities
+pg 4
+(Restricted cash $2.6bn sits in prepaid expenses, not in cash - not added; pg 10)</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Notes payable and other borrowings, current
+pg 4</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Finance lease liabilities, current
+pg 19
+(Within other current liabilities, not in borrowings - Oracle AR May 26 pg 118)</t>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Operating lease liabilities, current
+pg 19</t>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Notes payable and other borrowings, non-current
+pg 4</t>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Finance lease liabilities, non-current
+pg 19
+(Within other non-current liabilities, not in borrowings - Oracle AR May 26 pg 118)</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Operating lease liabilities (non-current)
+pg 4</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle AR May 26
+Aggregate net liability (funded status) of defined benefit plans
+pg 144
+(Carry-forward - not disclosed in QR)</t>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Preferred stock - 6.50% Series D Mandatory Convertible Preferred Stock
+pg 4</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Noncontrolling interests
+pg 4</t>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0">
+      <text>
+        <t>Oracle QR Aug 26
+Shares of common stock outstanding as of September 7, 2026: 3,023,736,000 (in millions)
+pg 1</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -443,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -465,7 +564,11 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
@@ -482,7 +585,11 @@
           <t>BS Currency</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n"/>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
@@ -506,7 +613,10 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
+      <c r="B4" s="7">
+        <f>-36369-708</f>
+        <v/>
+      </c>
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
@@ -523,7 +633,9 @@
           <t>Short Term Debt</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
+      <c r="B5" s="7" t="n">
+        <v>7625</v>
+      </c>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n"/>
@@ -540,7 +652,9 @@
           <t>ST Financial Lease</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
+      <c r="B6" s="7" t="n">
+        <v>749</v>
+      </c>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="n"/>
@@ -557,7 +671,9 @@
           <t>ST Operating Lease</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
+      <c r="B7" s="7" t="n">
+        <v>4027</v>
+      </c>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="n"/>
@@ -574,7 +690,9 @@
           <t>Long Term Debt</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
+      <c r="B8" s="7" t="n">
+        <v>117712</v>
+      </c>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="n"/>
@@ -591,7 +709,9 @@
           <t>LT Financial Lease</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n"/>
+      <c r="B9" s="7" t="n">
+        <v>8436</v>
+      </c>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="3" t="n"/>
@@ -608,7 +728,9 @@
           <t>LT Operating Lease</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
+      <c r="B10" s="7" t="n">
+        <v>30594</v>
+      </c>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="n"/>
@@ -642,7 +764,9 @@
           <t>Pensions</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="7" t="n">
+        <v>256</v>
+      </c>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="3" t="n"/>
@@ -659,7 +783,9 @@
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="7" t="n">
+        <v>4954</v>
+      </c>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="3" t="n"/>
@@ -676,7 +802,9 @@
           <t>Minorities</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="7" t="n">
+        <v>424</v>
+      </c>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
@@ -693,7 +821,9 @@
           <t>Shares</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="7" t="n">
+        <v>3023.736</v>
+      </c>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="n"/>
@@ -1005,5 +1135,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Title notes 'Claude Analyst', size them to fit, add price from Yahoo
- Notes carry the Claude Analyst author and title line, and are sized from
  their text so the full content shows on hover (re-applied before every
  save because openpyxl drops note sizes on reload)
- update_price.py fills row 19 with the Yahoo Finance close for a date
- Oracle price set to the 25 Sep 2026 close of 137.10 USD

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012dLLbpnyoNB7T2efRSv67L
</commit_message>
<xml_diff>
--- a/templates/TradingComps.xlsx
+++ b/templates/TradingComps.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00;(#,##0.00);&quot;-&quot;"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -75,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -84,6 +85,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -163,12 +165,13 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author/>
+    <author>Claude Analyst</author>
   </authors>
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Cash and cash equivalents
 pg 4
 Marketable securities
@@ -178,14 +181,16 @@
     </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Notes payable and other borrowings, current
 pg 4</t>
       </text>
     </comment>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Finance lease liabilities, current
 pg 19
 (Within other current liabilities, not in borrowings - Oracle AR May 26 pg 118)</t>
@@ -193,21 +198,24 @@
     </comment>
     <comment ref="B7" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Operating lease liabilities, current
 pg 19</t>
       </text>
     </comment>
     <comment ref="B8" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Notes payable and other borrowings, non-current
 pg 4</t>
       </text>
     </comment>
     <comment ref="B9" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Finance lease liabilities, non-current
 pg 19
 (Within other non-current liabilities, not in borrowings - Oracle AR May 26 pg 118)</t>
@@ -215,14 +223,16 @@
     </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Operating lease liabilities (non-current)
 pg 4</t>
       </text>
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">
       <text>
-        <t>Oracle AR May 26
+        <t>Claude Analyst:
+Oracle AR May 26
 Aggregate net liability (funded status) of defined benefit plans
 pg 144
 (Carry-forward - not disclosed in QR)</t>
@@ -230,23 +240,34 @@
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Preferred stock - 6.50% Series D Mandatory Convertible Preferred Stock
 pg 4</t>
       </text>
     </comment>
     <comment ref="B14" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Noncontrolling interests
 pg 4</t>
       </text>
     </comment>
     <comment ref="B16" authorId="0" shapeId="0">
       <text>
-        <t>Oracle QR Aug 26
+        <t>Claude Analyst:
+Oracle QR Aug 26
 Shares of common stock outstanding as of September 7, 2026: 3,023,736,000 (in millions)
 pg 1</t>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0">
+      <text>
+        <t>Claude Analyst:
+Yahoo Finance
+ORCL closing price (USD), 25 Sep 2026
+finance.yahoo.com/quote/ORCL/history</t>
       </text>
     </comment>
   </commentList>
@@ -542,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -815,6 +836,7 @@
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="n"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
@@ -834,6 +856,7 @@
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="n"/>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
@@ -887,7 +910,9 @@
           <t>Price</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
+      <c r="B19" s="8" t="n">
+        <v>137.1</v>
+      </c>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
@@ -945,6 +970,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Make the Claude Analyst note title bold
openpyxl only writes plain-text notes, so after each save the note XML is
rewritten as a bold title run plus a regular body run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012dLLbpnyoNB7T2efRSv67L
</commit_message>
<xml_diff>
--- a/templates/TradingComps.xlsx
+++ b/templates/TradingComps.xlsx
@@ -170,104 +170,320 @@
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Cash and cash equivalents
 pg 4
 Marketable securities
 pg 4
 (Restricted cash $2.6bn sits in prepaid expenses, not in cash - not added; pg 10)</t>
+        </r>
       </text>
     </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Notes payable and other borrowings, current
 pg 4</t>
+        </r>
       </text>
     </comment>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Finance lease liabilities, current
 pg 19
 (Within other current liabilities, not in borrowings - Oracle AR May 26 pg 118)</t>
+        </r>
       </text>
     </comment>
     <comment ref="B7" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Operating lease liabilities, current
 pg 19</t>
+        </r>
       </text>
     </comment>
     <comment ref="B8" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Notes payable and other borrowings, non-current
 pg 4</t>
+        </r>
       </text>
     </comment>
     <comment ref="B9" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Finance lease liabilities, non-current
 pg 19
 (Within other non-current liabilities, not in borrowings - Oracle AR May 26 pg 118)</t>
+        </r>
       </text>
     </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Operating lease liabilities (non-current)
 pg 4</t>
+        </r>
       </text>
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle AR May 26
 Aggregate net liability (funded status) of defined benefit plans
 pg 144
 (Carry-forward - not disclosed in QR)</t>
+        </r>
       </text>
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Preferred stock - 6.50% Series D Mandatory Convertible Preferred Stock
 pg 4</t>
+        </r>
       </text>
     </comment>
     <comment ref="B14" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Noncontrolling interests
 pg 4</t>
+        </r>
       </text>
     </comment>
     <comment ref="B16" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Oracle QR Aug 26
 Shares of common stock outstanding as of September 7, 2026: 3,023,736,000 (in millions)
 pg 1</t>
+        </r>
       </text>
     </comment>
     <comment ref="B19" authorId="0" shapeId="0">
       <text>
-        <t>Claude Analyst:
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Claude Analyst:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Yahoo Finance
 ORCL closing price (USD), 25 Sep 2026
 finance.yahoo.com/quote/ORCL/history</t>
+        </r>
       </text>
     </comment>
   </commentList>

</xml_diff>